<commit_message>
Grouped videos by category
</commit_message>
<xml_diff>
--- a/frontend/Video Database.xlsx
+++ b/frontend/Video Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jasminerojas/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="189" documentId="8_{098F0E94-7DCA-D542-868A-C2B6A23371D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AA4D55B5-CFBB-4AAD-92E0-86963B4AF315}"/>
+  <xr:revisionPtr revIDLastSave="255" documentId="8_{098F0E94-7DCA-D542-868A-C2B6A23371D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64F682E7-D0A4-4190-8B8F-2FF5A407DB86}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="600" windowWidth="23660" windowHeight="14320" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="600" windowWidth="23660" windowHeight="14320" firstSheet="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Healthy Lifestyle Edu Videos" sheetId="6" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="131">
   <si>
     <t>Video Title</t>
   </si>
@@ -62,6 +62,21 @@
     <t>American Heart Association</t>
   </si>
   <si>
+    <t>Exploring Low-Cost Healthy Resources</t>
+  </si>
+  <si>
+    <t>https://youtu.be/24NNKYxqcNc?si=YcSrO4g0WUzeuH6c</t>
+  </si>
+  <si>
+    <t>How to Health UF</t>
+  </si>
+  <si>
+    <t>How to Read a Nutrition Label</t>
+  </si>
+  <si>
+    <t>https://youtu.be/43u6GWlsmto?si=85Mc4VfmRAgWelbR</t>
+  </si>
+  <si>
     <t>Life's Essential 8: The Checklist for Lifelong Good Health</t>
   </si>
   <si>
@@ -80,6 +95,18 @@
     <t>https://youtu.be/7Z0CaNLXxpo?si=ulT2JwHQba2PKBdp </t>
   </si>
   <si>
+    <t>Healthy Ingredient Swap</t>
+  </si>
+  <si>
+    <t>https://youtu.be/nz24KFGgCoo?si=GWT4yfh8g5pp7LKr</t>
+  </si>
+  <si>
+    <t>Healthy Holiday Swaps</t>
+  </si>
+  <si>
+    <t>https://youtu.be/8B2mf9URhyY?si=AXHdNZqf-mvp8epa</t>
+  </si>
+  <si>
     <t>Recipe Title</t>
   </si>
   <si>
@@ -131,6 +158,24 @@
     <t>https://youtu.be/cVzzfnD6Nho?si=jRrdN4YMpCmVrFFw</t>
   </si>
   <si>
+    <t>Grilled Cuban Mojo Marinated Pork Tenderloin with Fried Plantains</t>
+  </si>
+  <si>
+    <t>https://youtu.be/tlETbw9mghg?si=h-DT1YtnZmhV8XND</t>
+  </si>
+  <si>
+    <t>Grilled Lemon Garlic Chicken with Grilled Okra Recipe</t>
+  </si>
+  <si>
+    <t>https://youtu.be/dNMKsHYYJxk?si=0lwux16mRhsJ3ZmI</t>
+  </si>
+  <si>
+    <t>Haitian Pork Griot</t>
+  </si>
+  <si>
+    <t>https://youtu.be/k1w_u3U4Rtk?si=eQ77U57HMMUl-WuX</t>
+  </si>
+  <si>
     <t>Oatmeal Zucchini Bars</t>
   </si>
   <si>
@@ -161,6 +206,12 @@
     <t>https://youtu.be/dxuZroN4Hgo?si=r5YWiTmPCVyon7Lm</t>
   </si>
   <si>
+    <t>Sweet and Sour Pork Fried Rice</t>
+  </si>
+  <si>
+    <t>https://youtu.be/zBgVVG0pKEg?si=Gs7dlfEqqPFqkY1h</t>
+  </si>
+  <si>
     <t>Tofu Banh Mi Noodle Bowls</t>
   </si>
   <si>
@@ -173,6 +224,15 @@
     <t>https://youtu.be/ROd0LC-j79M?si=u_tar4rg1-IjK2XP</t>
   </si>
   <si>
+    <t>DASH Diet</t>
+  </si>
+  <si>
+    <t>https://youtu.be/aF1jlW6uXDo?si=-ZXdcdZP99tGqn15</t>
+  </si>
+  <si>
+    <t>UF IFAS Social</t>
+  </si>
+  <si>
     <t>DASH Recommendations</t>
   </si>
   <si>
@@ -182,6 +242,18 @@
     <t>Penn State Excursion</t>
   </si>
   <si>
+    <t>Dietary Guide for Managing 'Hypertension' or 'High blood pressure'</t>
+  </si>
+  <si>
+    <t>https://youtu.be/LYSINC9aLuM?si=LQuRgvikhho8iq3q</t>
+  </si>
+  <si>
+    <t>How Much Sodium Should You Eat Per Day?</t>
+  </si>
+  <si>
+    <t>https://youtu.be/0lUYfyLKxDU?si=L_9l6AeK15wqYs_x</t>
+  </si>
+  <si>
     <t>How to Monitor Your Blood Pressure at Home</t>
   </si>
   <si>
@@ -215,6 +287,12 @@
     <t>https://youtu.be/MEhcdMcvlfM?si=Q8KsSnlOFkgHZFhf </t>
   </si>
   <si>
+    <t>What is Cholesterol?</t>
+  </si>
+  <si>
+    <t>https://youtu.be/UaolDzxn-vE?si=uNYsfAncuzt3L5wg</t>
+  </si>
+  <si>
     <t xml:space="preserve">Diabetes- and Kidney-Friendly Roasted Chicken with Veggies and Cranberries </t>
   </si>
   <si>
@@ -257,6 +335,24 @@
     <t>American Association of Clinical Endocrinology</t>
   </si>
   <si>
+    <t>Diabetes and Beverages</t>
+  </si>
+  <si>
+    <t>https://youtu.be/I4lPcKhTED8?si=fJyTjIF0T-n8TZqv</t>
+  </si>
+  <si>
+    <t>Diabetes MyPlate Method</t>
+  </si>
+  <si>
+    <t>https://youtu.be/IszLpEwZqyI?si=WOCauMTajmtQvffs</t>
+  </si>
+  <si>
+    <t>Dietary Guide for Managing Diabetes</t>
+  </si>
+  <si>
+    <t>https://youtu.be/GZduv-Akky4?si=LFQy10xqSQ7dvq-F</t>
+  </si>
+  <si>
     <t>Food and Your Health: Blood Sugar</t>
   </si>
   <si>
@@ -266,6 +362,21 @@
     <t>American Heart Associaiton</t>
   </si>
   <si>
+    <t>Foods that Don't Raise Blood Sugar</t>
+  </si>
+  <si>
+    <t>https://youtu.be/U3YQPlsZcqg?si=VlmwWidQvgTiKfbw</t>
+  </si>
+  <si>
+    <t>How Much Sugar is in Your Soft Drink?</t>
+  </si>
+  <si>
+    <t>https://youtu.be/ZeV8s1FDmFY?si=dFiSAzjXAKMaB4Ei</t>
+  </si>
+  <si>
+    <t>UF Health Jacksonville</t>
+  </si>
+  <si>
     <t>How to Pack Your Diabetes Emergency Kit</t>
   </si>
   <si>
@@ -302,6 +413,12 @@
     <t>https://youtu.be/0PBGnEgkXH4?si=DGptgBkBn3Nwes3t</t>
   </si>
   <si>
+    <t>Papas Fritas en Fridora de Aire</t>
+  </si>
+  <si>
+    <t>https://youtu.be/HAfB2GwvwFQ?si=TgzkyS1u3_3-9iSv</t>
+  </si>
+  <si>
     <t>Plátanos Fritos en Freidora de Aire con Crema de Cilantro</t>
   </si>
   <si>
@@ -318,12 +435,6 @@
   </si>
   <si>
     <t>https://youtu.be/_-5zi2T8LBk?si=di2Ba_sJB32Lj0b5</t>
-  </si>
-  <si>
-    <t>Papas Fritas en Fridora de Aire</t>
-  </si>
-  <si>
-    <t>https://youtu.be/HAfB2GwvwFQ?si=TgzkyS1u3_3-9iSv</t>
   </si>
 </sst>
 </file>
@@ -704,7 +815,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94BB0CA9-C7A6-4793-AA8F-625FD2340D25}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -742,40 +853,88 @@
         <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
         <v>8</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
       </c>
     </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C5">
-    <sortCondition ref="A2:A5"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C7">
+    <sortCondition ref="A2:A7"/>
   </sortState>
   <hyperlinks>
-    <hyperlink ref="B3" r:id="rId1" xr:uid="{B4134850-8FC2-4745-8B33-CB24747A0950}"/>
+    <hyperlink ref="B5" r:id="rId1" xr:uid="{B4134850-8FC2-4745-8B33-CB24747A0950}"/>
     <hyperlink ref="B2" r:id="rId2" xr:uid="{FF2003AD-AEC8-421C-AEB0-535DE79CD205}"/>
-    <hyperlink ref="B5" r:id="rId3" xr:uid="{32611D62-80C8-47CE-BD28-835BF3765540}"/>
-    <hyperlink ref="B4" r:id="rId4" xr:uid="{45D38A21-9577-46A2-B423-91235310A18E}"/>
+    <hyperlink ref="B7" r:id="rId3" xr:uid="{32611D62-80C8-47CE-BD28-835BF3765540}"/>
+    <hyperlink ref="B6" r:id="rId4" xr:uid="{45D38A21-9577-46A2-B423-91235310A18E}"/>
+    <hyperlink ref="B4" r:id="rId5" xr:uid="{6F74B7CE-BEDA-4258-B37F-B152CD5E5D2F}"/>
+    <hyperlink ref="B3" r:id="rId6" xr:uid="{624E9155-11E3-4C05-9843-19C0411BA390}"/>
+    <hyperlink ref="B8" r:id="rId7" xr:uid="{0E5A786B-EA37-4DCA-B82F-C1917BF8D43B}"/>
+    <hyperlink ref="B9" r:id="rId8" xr:uid="{CF078E1D-BF65-4057-82CA-74B3BF804943}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -783,20 +942,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49FC47DB-EBDE-4E16-9777-A05BA959AFBE}">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="44.42578125" customWidth="1"/>
+    <col min="1" max="1" width="59.85546875" customWidth="1"/>
     <col min="2" max="2" width="52.140625" customWidth="1"/>
     <col min="3" max="3" width="41" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="3" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>2</v>
@@ -804,10 +963,10 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="C2" t="s">
         <v>5</v>
@@ -815,10 +974,10 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="C3" t="s">
         <v>5</v>
@@ -826,10 +985,10 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
         <v>5</v>
@@ -837,10 +996,10 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
@@ -848,21 +1007,21 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="C7" t="s">
         <v>5</v>
@@ -870,21 +1029,21 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="C9" t="s">
         <v>5</v>
@@ -892,10 +1051,10 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>32</v>
+        <v>40</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="C10" t="s">
         <v>5</v>
@@ -903,10 +1062,10 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="C11" t="s">
         <v>5</v>
@@ -914,10 +1073,10 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="C12" t="s">
         <v>5</v>
@@ -925,10 +1084,10 @@
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>37</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>38</v>
+        <v>46</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>47</v>
       </c>
       <c r="C13" t="s">
         <v>5</v>
@@ -936,10 +1095,10 @@
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="C14" t="s">
         <v>5</v>
@@ -947,34 +1106,82 @@
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="C15" t="s">
-        <v>24</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
+        <v>54</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" t="s">
+        <v>56</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" t="s">
+        <v>58</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C19" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C15">
-    <sortCondition ref="A2:A15"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C19">
+    <sortCondition ref="A2:A19"/>
   </sortState>
   <hyperlinks>
-    <hyperlink ref="B10" r:id="rId1" xr:uid="{49F98E03-AC64-41D8-AA36-760A3E0A1C85}"/>
-    <hyperlink ref="B9" r:id="rId2" xr:uid="{A37981C3-534E-4E8D-ADDB-9C9689564BF3}"/>
-    <hyperlink ref="B11" r:id="rId3" xr:uid="{FB76ADFB-4300-493E-B616-A100C387C018}"/>
+    <hyperlink ref="B13" r:id="rId1" xr:uid="{49F98E03-AC64-41D8-AA36-760A3E0A1C85}"/>
+    <hyperlink ref="B12" r:id="rId2" xr:uid="{A37981C3-534E-4E8D-ADDB-9C9689564BF3}"/>
+    <hyperlink ref="B14" r:id="rId3" xr:uid="{FB76ADFB-4300-493E-B616-A100C387C018}"/>
     <hyperlink ref="B4" r:id="rId4" xr:uid="{548072F5-544A-44D5-88F7-6BD67AA8B269}"/>
     <hyperlink ref="B5" r:id="rId5" xr:uid="{EF849BB5-7C95-4E9A-9DF1-1EFF9CE553AB}"/>
-    <hyperlink ref="B14" r:id="rId6" xr:uid="{6B622F30-CAFA-40A8-8457-A95386F0DA47}"/>
+    <hyperlink ref="B18" r:id="rId6" xr:uid="{6B622F30-CAFA-40A8-8457-A95386F0DA47}"/>
     <hyperlink ref="B8" r:id="rId7" xr:uid="{F8AE288C-82D3-4860-8968-C2966A532037}"/>
     <hyperlink ref="B6" r:id="rId8" xr:uid="{17036A1B-8E9E-42F2-A93C-1424FB522174}"/>
-    <hyperlink ref="B15" r:id="rId9" xr:uid="{BB295D7D-2A65-4375-B2B2-C3F63CD5D766}"/>
-    <hyperlink ref="B13" r:id="rId10" xr:uid="{79B9B206-8A22-475E-80B5-5B88AF871992}"/>
+    <hyperlink ref="B19" r:id="rId9" xr:uid="{BB295D7D-2A65-4375-B2B2-C3F63CD5D766}"/>
+    <hyperlink ref="B16" r:id="rId10" xr:uid="{79B9B206-8A22-475E-80B5-5B88AF871992}"/>
     <hyperlink ref="B3" r:id="rId11" xr:uid="{DF7A8330-5753-494A-B750-FC6405D3B3F7}"/>
     <hyperlink ref="B2" r:id="rId12" xr:uid="{40F846F4-6EBC-4A2C-BBCF-FADCFC97A9F2}"/>
     <hyperlink ref="B7" r:id="rId13" xr:uid="{41ECD1CD-D402-4E5C-8597-75D44E0F5DA6}"/>
-    <hyperlink ref="B12" r:id="rId14" xr:uid="{AFCB8587-B87E-4B75-87A2-EC5015A00ED4}"/>
+    <hyperlink ref="B15" r:id="rId14" xr:uid="{AFCB8587-B87E-4B75-87A2-EC5015A00ED4}"/>
+    <hyperlink ref="B11" r:id="rId15" xr:uid="{0698539C-6383-49A3-AF8E-E6F5D5828805}"/>
+    <hyperlink ref="B9" r:id="rId16" xr:uid="{53E250CE-05A2-43BF-8FE1-A487D6D67B92}"/>
+    <hyperlink ref="B17" r:id="rId17" xr:uid="{42B0F15A-51AB-46E0-BCBE-B5089638DCCD}"/>
+    <hyperlink ref="B10" r:id="rId18" xr:uid="{E3CF25E9-CE31-4DFA-BC95-648A84AA4331}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -982,10 +1189,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82E87408-0E2A-48C5-A3CF-6A23C8D1659C}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="44.42578125" customWidth="1"/>
+    <col min="1" max="1" width="59.42578125" customWidth="1"/>
     <col min="2" max="2" width="52.140625" customWidth="1"/>
     <col min="3" max="3" width="28.140625" customWidth="1"/>
   </cols>
@@ -1003,54 +1210,54 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="C2" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>47</v>
+        <v>64</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="C4" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="C5" t="s">
-        <v>52</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>54</v>
+      <c r="A6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>71</v>
       </c>
       <c r="C6" t="s">
         <v>5</v>
@@ -1058,29 +1265,74 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>56</v>
+        <v>73</v>
       </c>
       <c r="C7" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:3">
-      <c r="B8" s="1"/>
+      <c r="A8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C8" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C9" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C10" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>81</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C11" t="s">
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C8">
-    <sortCondition ref="A2:A8"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C11">
+    <sortCondition ref="A2:A11"/>
   </sortState>
   <hyperlinks>
-    <hyperlink ref="B7" r:id="rId1" xr:uid="{DDB1B95B-666D-4B9B-8888-E80A7849FEDB}"/>
-    <hyperlink ref="B3" r:id="rId2" xr:uid="{2821DBFD-1517-4C01-A54D-F0DD19916BDB}"/>
-    <hyperlink ref="B4" r:id="rId3" xr:uid="{76BFE417-0FF2-41A3-B065-7579EA0DAF65}"/>
-    <hyperlink ref="B6" r:id="rId4" xr:uid="{4669B4F9-99B8-4648-91F6-B807C778F5BC}"/>
-    <hyperlink ref="B2" r:id="rId5" xr:uid="{5D5AFACB-4EBD-4D0C-9C53-4648BB0A9C48}"/>
-    <hyperlink ref="B5" r:id="rId6" xr:uid="{1DD9C612-6768-4319-AEED-CE5A621FD68C}"/>
+    <hyperlink ref="B10" r:id="rId1" xr:uid="{DDB1B95B-666D-4B9B-8888-E80A7849FEDB}"/>
+    <hyperlink ref="B6" r:id="rId2" xr:uid="{2821DBFD-1517-4C01-A54D-F0DD19916BDB}"/>
+    <hyperlink ref="B7" r:id="rId3" xr:uid="{76BFE417-0FF2-41A3-B065-7579EA0DAF65}"/>
+    <hyperlink ref="B9" r:id="rId4" xr:uid="{4669B4F9-99B8-4648-91F6-B807C778F5BC}"/>
+    <hyperlink ref="B3" r:id="rId5" xr:uid="{5D5AFACB-4EBD-4D0C-9C53-4648BB0A9C48}"/>
+    <hyperlink ref="B8" r:id="rId6" xr:uid="{1DD9C612-6768-4319-AEED-CE5A621FD68C}"/>
+    <hyperlink ref="B11" r:id="rId7" xr:uid="{AC0B49A4-C981-42B3-BFE9-65207FA3DE5D}"/>
+    <hyperlink ref="B2" r:id="rId8" xr:uid="{A6692115-17F9-441E-BB5D-462ABAF073D9}"/>
+    <hyperlink ref="B4" r:id="rId9" xr:uid="{3BD1C8F2-F54C-41A1-A59B-7D621D133860}"/>
+    <hyperlink ref="B5" r:id="rId10" xr:uid="{6530A4EF-EED9-49B4-93BF-593EBB6B6CC0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1098,10 +1350,10 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="3" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>2</v>
@@ -1109,57 +1361,57 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>57</v>
+        <v>83</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>58</v>
+        <v>84</v>
       </c>
       <c r="C2" t="s">
-        <v>59</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="4" t="s">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>61</v>
+        <v>87</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>59</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>62</v>
+        <v>88</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>63</v>
+        <v>89</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>65</v>
+        <v>91</v>
       </c>
       <c r="C5" t="s">
-        <v>59</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>67</v>
+        <v>93</v>
       </c>
       <c r="C6" t="s">
-        <v>59</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -1200,69 +1452,117 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>68</v>
+        <v>94</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>69</v>
+        <v>95</v>
       </c>
       <c r="C2" t="s">
-        <v>70</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>71</v>
+        <v>97</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>72</v>
+        <v>98</v>
       </c>
       <c r="C3" t="s">
-        <v>73</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>99</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="C4" t="s">
-        <v>70</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>76</v>
+        <v>101</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>77</v>
+        <v>102</v>
       </c>
       <c r="C5" t="s">
-        <v>70</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C6" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="B7" s="1"/>
+      <c r="A7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C7" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="8" spans="1:3">
-      <c r="B8" s="1"/>
+      <c r="A8" t="s">
+        <v>108</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C8" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="9" spans="1:3">
-      <c r="B9" s="1"/>
+      <c r="A9" t="s">
+        <v>111</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C9" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="10" spans="1:3">
-      <c r="B10" s="1"/>
+      <c r="A10" t="s">
+        <v>113</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C10" t="s">
+        <v>96</v>
+      </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C10">
     <sortCondition ref="A2:A10"/>
   </sortState>
   <hyperlinks>
-    <hyperlink ref="B3" r:id="rId1" xr:uid="{B1624874-01B6-4276-9432-55F3C67CD6A6}"/>
-    <hyperlink ref="B5" r:id="rId2" xr:uid="{E9187404-58C1-4888-AF77-6CCF7763EC79}"/>
+    <hyperlink ref="B6" r:id="rId1" xr:uid="{B1624874-01B6-4276-9432-55F3C67CD6A6}"/>
+    <hyperlink ref="B10" r:id="rId2" xr:uid="{E9187404-58C1-4888-AF77-6CCF7763EC79}"/>
     <hyperlink ref="B2" r:id="rId3" xr:uid="{3236BBBE-B771-4CAB-A218-F78B33F91040}"/>
-    <hyperlink ref="B4" r:id="rId4" xr:uid="{410F3C31-5838-497B-AC23-662C1EC31172}"/>
+    <hyperlink ref="B9" r:id="rId4" xr:uid="{410F3C31-5838-497B-AC23-662C1EC31172}"/>
+    <hyperlink ref="B8" r:id="rId5" xr:uid="{BB8B7EC3-67AA-4C49-96E9-093DF04352A3}"/>
+    <hyperlink ref="B5" r:id="rId6" xr:uid="{B2EF8A6C-8A53-432A-9E83-CB63132F1676}"/>
+    <hyperlink ref="B3" r:id="rId7" xr:uid="{4DCF9635-9B2D-4FF0-B2E0-9CEF37CE8DB5}"/>
+    <hyperlink ref="B7" r:id="rId8" xr:uid="{81D980F3-03D1-4655-853F-BAFB516E24C2}"/>
+    <hyperlink ref="B4" r:id="rId9" xr:uid="{B3E4EBDB-5F78-40A5-B4DA-53159DB70772}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1280,10 +1580,10 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="3" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>2</v>
@@ -1291,10 +1591,10 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>78</v>
+        <v>115</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>79</v>
+        <v>116</v>
       </c>
       <c r="C2" t="s">
         <v>5</v>
@@ -1302,10 +1602,10 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>80</v>
+        <v>117</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>81</v>
+        <v>118</v>
       </c>
       <c r="C3" t="s">
         <v>5</v>
@@ -1313,10 +1613,10 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>82</v>
+        <v>119</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>83</v>
+        <v>120</v>
       </c>
       <c r="C4" t="s">
         <v>5</v>
@@ -1324,10 +1624,10 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>84</v>
+        <v>121</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>85</v>
+        <v>122</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
@@ -1335,10 +1635,10 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>123</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>87</v>
+        <v>124</v>
       </c>
       <c r="C6" t="s">
         <v>5</v>
@@ -1346,10 +1646,10 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>88</v>
+        <v>125</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>89</v>
+        <v>126</v>
       </c>
       <c r="C7" t="s">
         <v>5</v>
@@ -1357,10 +1657,10 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>90</v>
+        <v>127</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>91</v>
+        <v>128</v>
       </c>
       <c r="C8" t="s">
         <v>5</v>
@@ -1368,10 +1668,10 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>92</v>
+        <v>129</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="C9" t="s">
         <v>5</v>
@@ -1403,11 +1703,11 @@
     <hyperlink ref="B5" r:id="rId1" xr:uid="{D1C6E97A-6FAA-4219-9C36-EC9BDF3BE5DD}"/>
     <hyperlink ref="B3" r:id="rId2" xr:uid="{A7808F27-B70F-4E31-B4C0-29C19B8778C6}"/>
     <hyperlink ref="B2" r:id="rId3" xr:uid="{F94C5A55-9032-4CA8-9CA6-6586CBF457D1}"/>
-    <hyperlink ref="B7" r:id="rId4" xr:uid="{894392F2-10DC-4C74-BA3D-3CD7065000A6}"/>
+    <hyperlink ref="B8" r:id="rId4" xr:uid="{894392F2-10DC-4C74-BA3D-3CD7065000A6}"/>
     <hyperlink ref="B4" r:id="rId5" xr:uid="{B8FABC74-9E4A-4329-9F6B-E38BC071E8A0}"/>
-    <hyperlink ref="B8" r:id="rId6" xr:uid="{D8F95679-BA6C-4126-8642-2B87160D6FED}"/>
-    <hyperlink ref="B6" r:id="rId7" xr:uid="{FDF11205-FB65-4FE4-B919-6802ECE8F564}"/>
-    <hyperlink ref="B9" r:id="rId8" xr:uid="{FC9D4109-8521-4503-90C7-FE239C860E70}"/>
+    <hyperlink ref="B9" r:id="rId6" xr:uid="{D8F95679-BA6C-4126-8642-2B87160D6FED}"/>
+    <hyperlink ref="B7" r:id="rId7" xr:uid="{FDF11205-FB65-4FE4-B919-6802ECE8F564}"/>
+    <hyperlink ref="B6" r:id="rId8" xr:uid="{FC9D4109-8521-4503-90C7-FE239C860E70}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>